<commit_message>
coal retirement eco sensi
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/SuppXLS/Scen_Par-ETSAP_CT.xlsx
+++ b/VerveStacks_ZAF_grids_kan/SuppXLS/Scen_Par-ETSAP_CT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\VerveStacks_ZAF_grids_kan\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A34ED71-C666-437A-B69B-5D2835A13E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF40DA37-5777-4189-9114-1F5B94DA040C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
     <sheet name="ar6_r10" sheetId="3" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Veda!$B$8:$H$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Veda!$C$8:$H$136</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -102,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1703" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1774" uniqueCount="165">
   <si>
     <t>C1</t>
   </si>
@@ -578,7 +578,25 @@
     <t>NCAP_ELIFE</t>
   </si>
   <si>
-    <t>1-64</t>
+    <t>CoaRet</t>
+  </si>
+  <si>
+    <t>Pln</t>
+  </si>
+  <si>
+    <t>Eco</t>
+  </si>
+  <si>
+    <t>NCAP_TLIFE</t>
+  </si>
+  <si>
+    <t>+25</t>
+  </si>
+  <si>
+    <t>pset_pn</t>
+  </si>
+  <si>
+    <t>ep_coal_sub*,-*rf</t>
   </si>
 </sst>
 </file>
@@ -786,7 +804,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -823,6 +841,9 @@
     <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -993,22 +1014,22 @@
                   <c:v>229.26</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>242.36057142857143</c:v>
+                  <c:v>275.11199999999997</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>246.61825714285717</c:v>
+                  <c:v>290.01390000000004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>250.87594285714286</c:v>
+                  <c:v>304.91579999999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>270.52679999999998</c:v>
+                  <c:v>373.69379999999995</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>294.76285714285711</c:v>
+                  <c:v>458.52</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>315.85477714285713</c:v>
+                  <c:v>532.34172000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1284,19 +1305,19 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>35</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>60</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>80</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>95</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5885,7 +5906,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR78"/>
+  <dimension ref="A1:AR136"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="6.46484375" bestFit="1" customWidth="1"/>
@@ -5895,7 +5916,7 @@
     <col min="5" max="5" width="7.73046875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.1328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="3.86328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="3.86328125" customWidth="1"/>
+    <col min="8" max="8" width="6.59765625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="1.73046875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="24.53125" customWidth="1"/>
@@ -5916,14 +5937,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.45">
-      <c r="K1" s="16" t="s">
-        <v>158</v>
+      <c r="K1" s="16">
+        <v>65</v>
+      </c>
+      <c r="L1">
+        <v>66</v>
+      </c>
+      <c r="M1">
+        <v>67</v>
+      </c>
+      <c r="N1">
+        <v>68</v>
+      </c>
+      <c r="O1">
+        <v>73</v>
+      </c>
+      <c r="P1">
+        <v>74</v>
+      </c>
+      <c r="Q1">
+        <v>75</v>
+      </c>
+      <c r="R1">
+        <v>76</v>
+      </c>
+      <c r="S1">
+        <v>81</v>
+      </c>
+      <c r="T1">
+        <v>82</v>
+      </c>
+      <c r="U1">
+        <v>83</v>
+      </c>
+      <c r="V1">
+        <v>84</v>
+      </c>
+      <c r="W1">
+        <v>89</v>
+      </c>
+      <c r="X1">
+        <v>90</v>
+      </c>
+      <c r="Y1">
+        <v>91</v>
+      </c>
+      <c r="Z1">
+        <v>92</v>
+      </c>
+      <c r="AA1">
+        <v>97</v>
+      </c>
+      <c r="AB1">
+        <v>98</v>
+      </c>
+      <c r="AC1">
+        <v>99</v>
+      </c>
+      <c r="AD1">
+        <v>100</v>
+      </c>
+      <c r="AE1">
+        <v>105</v>
+      </c>
+      <c r="AF1">
+        <v>106</v>
+      </c>
+      <c r="AG1">
+        <v>107</v>
+      </c>
+      <c r="AH1">
+        <v>108</v>
+      </c>
+      <c r="AI1">
+        <v>113</v>
+      </c>
+      <c r="AJ1">
+        <v>114</v>
+      </c>
+      <c r="AK1">
+        <v>115</v>
+      </c>
+      <c r="AL1">
+        <v>116</v>
+      </c>
+      <c r="AM1">
+        <v>121</v>
+      </c>
+      <c r="AN1">
+        <v>122</v>
+      </c>
+      <c r="AO1">
+        <v>123</v>
+      </c>
+      <c r="AP1">
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:44" x14ac:dyDescent="0.45">
       <c r="B2" s="1" t="str">
         <f>"~Inputcell: "&amp;_xlfn.TEXTJOIN(",",TRUE,K1:EI1)</f>
-        <v>~Inputcell: 1-64</v>
+        <v>~Inputcell: 65,66,67,68,73,74,75,76,81,82,83,84,89,90,91,92,97,98,99,100,105,106,107,108,113,114,115,116,121,122,123,124</v>
       </c>
       <c r="L2" t="s">
         <v>131</v>
@@ -5956,7 +6070,7 @@
     </row>
     <row r="3" spans="1:44" x14ac:dyDescent="0.45">
       <c r="B3" s="9">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="L3" t="s">
         <v>133</v>
@@ -5992,11 +6106,11 @@
     <row r="5" spans="1:44" x14ac:dyDescent="0.45">
       <c r="D5" s="21" t="str">
         <f t="shared" ref="D5:I5" si="1">VLOOKUP($B$3,$C$9:$K$999,COLUMN()-2,FALSE)</f>
-        <v>Lo</v>
+        <v>Hi</v>
       </c>
       <c r="E5" s="21">
         <f t="shared" si="1"/>
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="F5" s="21" t="str">
         <f t="shared" si="1"/>
@@ -6004,11 +6118,11 @@
       </c>
       <c r="G5" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="H5" s="21" t="str">
         <f t="shared" si="1"/>
-        <v>Y</v>
+        <v>Eco</v>
       </c>
       <c r="I5" s="21">
         <f t="shared" si="1"/>
@@ -6093,7 +6207,7 @@
         <v>134</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>152</v>
@@ -6109,7 +6223,7 @@
       </c>
       <c r="B9" t="str">
         <f>_xlfn.TEXTJOIN(".",TRUE,D9:I9)</f>
-        <v>Lo.0.CF1.Y.Y.1</v>
+        <v>Lo.0.CF1.Y.Pln.1</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -6127,7 +6241,7 @@
         <v>135</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I9" s="22">
         <v>1</v>
@@ -6154,7 +6268,7 @@
       </c>
       <c r="B10" t="str">
         <f t="shared" ref="B10:B56" si="2">_xlfn.TEXTJOIN(".",TRUE,D10:I10)</f>
-        <v>Hi.0.CF1.Y.Y.1</v>
+        <v>Hi.0.CF1.Y.Pln.1</v>
       </c>
       <c r="C10">
         <f>C9+1</f>
@@ -6173,7 +6287,7 @@
         <v>135</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I10" s="22">
         <v>1</v>
@@ -6203,10 +6317,10 @@
       </c>
       <c r="B11" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF1.Y.Y.1</v>
+        <v>Lo.95.CF1.Y.Pln.1</v>
       </c>
       <c r="C11">
-        <f t="shared" ref="C11:C72" si="3">C10+1</f>
+        <f t="shared" ref="C11:C74" si="3">C10+1</f>
         <v>3</v>
       </c>
       <c r="D11" t="str">
@@ -6223,7 +6337,7 @@
         <v>135</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I11" s="22">
         <v>1</v>
@@ -6253,14 +6367,14 @@
       </c>
       <c r="B12" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF1.Y.Y.1</v>
+        <v>Hi.95.CF1.Y.Pln.1</v>
       </c>
       <c r="C12">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
       <c r="D12" t="str">
-        <f t="shared" ref="D12:D72" si="4">D10</f>
+        <f t="shared" ref="D12:D75" si="4">D10</f>
         <v>Hi</v>
       </c>
       <c r="E12">
@@ -6273,7 +6387,7 @@
         <v>135</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I12" s="22">
         <v>1</v>
@@ -6307,7 +6421,7 @@
       </c>
       <c r="B13" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF1.N.Y.1</v>
+        <v>Lo.0.CF1.N.Pln.1</v>
       </c>
       <c r="C13">
         <f t="shared" si="3"/>
@@ -6328,7 +6442,7 @@
         <v>136</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I13" s="22">
         <v>1</v>
@@ -6355,7 +6469,7 @@
       </c>
       <c r="B14" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF1.N.Y.1</v>
+        <v>Hi.0.CF1.N.Pln.1</v>
       </c>
       <c r="C14">
         <f t="shared" si="3"/>
@@ -6376,7 +6490,7 @@
         <v>136</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I14" s="22">
         <v>1</v>
@@ -6387,27 +6501,27 @@
       </c>
       <c r="Y14" s="8">
         <f t="shared" ref="Y14:AD14" si="6">$W$12*N15</f>
-        <v>242.36057142857143</v>
+        <v>275.11199999999997</v>
       </c>
       <c r="Z14" s="8">
         <f t="shared" si="6"/>
-        <v>246.61825714285717</v>
+        <v>290.01390000000004</v>
       </c>
       <c r="AA14" s="8">
         <f t="shared" si="6"/>
-        <v>250.87594285714286</v>
+        <v>304.91579999999999</v>
       </c>
       <c r="AB14" s="8">
         <f t="shared" si="6"/>
-        <v>270.52679999999998</v>
+        <v>373.69379999999995</v>
       </c>
       <c r="AC14" s="8">
         <f t="shared" si="6"/>
-        <v>294.76285714285711</v>
+        <v>458.52</v>
       </c>
       <c r="AD14" s="8">
         <f t="shared" si="6"/>
-        <v>315.85477714285713</v>
+        <v>532.34172000000001</v>
       </c>
       <c r="AN14" s="10">
         <f>AN9+1</f>
@@ -6420,7 +6534,7 @@
       </c>
       <c r="B15" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF1.N.Y.1</v>
+        <v>Lo.95.CF1.N.Pln.1</v>
       </c>
       <c r="C15">
         <f t="shared" si="3"/>
@@ -6441,7 +6555,7 @@
         <v>136</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I15" s="22">
         <v>1</v>
@@ -6455,27 +6569,27 @@
       </c>
       <c r="N15" s="11">
         <f t="shared" si="8"/>
-        <v>1.0571428571428572</v>
+        <v>1.2</v>
       </c>
       <c r="O15" s="11">
         <f t="shared" si="8"/>
-        <v>1.0757142857142858</v>
+        <v>1.2650000000000001</v>
       </c>
       <c r="P15" s="11">
         <f t="shared" si="8"/>
-        <v>1.0942857142857143</v>
+        <v>1.33</v>
       </c>
       <c r="Q15" s="11">
         <f t="shared" si="8"/>
-        <v>1.18</v>
+        <v>1.63</v>
       </c>
       <c r="R15" s="11">
         <f t="shared" si="8"/>
-        <v>1.2857142857142856</v>
+        <v>2</v>
       </c>
       <c r="S15" s="11">
         <f t="shared" si="8"/>
-        <v>1.3777142857142857</v>
+        <v>2.3220000000000001</v>
       </c>
       <c r="AN15" s="10">
         <f t="shared" ref="AN15:AN78" si="9">AN10+1</f>
@@ -6488,7 +6602,7 @@
       </c>
       <c r="B16" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF1.N.Y.1</v>
+        <v>Hi.95.CF1.N.Pln.1</v>
       </c>
       <c r="C16">
         <f t="shared" si="3"/>
@@ -6509,7 +6623,7 @@
         <v>136</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I16" s="22">
         <v>1</v>
@@ -6528,7 +6642,7 @@
       </c>
       <c r="B17" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF6.Y.Y.1</v>
+        <v>Lo.0.CF6.Y.Pln.1</v>
       </c>
       <c r="C17">
         <f t="shared" si="3"/>
@@ -6550,7 +6664,7 @@
         <v>Y</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I17" s="22">
         <v>1</v>
@@ -6623,7 +6737,7 @@
       </c>
       <c r="B18" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF6.Y.Y.1</v>
+        <v>Hi.0.CF6.Y.Pln.1</v>
       </c>
       <c r="C18">
         <f t="shared" si="3"/>
@@ -6641,11 +6755,11 @@
         <v>130</v>
       </c>
       <c r="G18" t="str">
-        <f t="shared" ref="G18:G72" si="14">G10</f>
+        <f t="shared" ref="G18:G81" si="14">G10</f>
         <v>Y</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I18" s="22">
         <v>1</v>
@@ -6706,11 +6820,11 @@
       </c>
       <c r="AC18" s="6">
         <f t="shared" si="15"/>
-        <v>2.947628571428571</v>
+        <v>4.5851999999999995</v>
       </c>
       <c r="AD18" s="6">
         <f t="shared" si="15"/>
-        <v>3.1585477714285712</v>
+        <v>5.3234172000000006</v>
       </c>
       <c r="AE18" t="s">
         <v>17</v>
@@ -6727,7 +6841,7 @@
       </c>
       <c r="B19" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF6.Y.Y.1</v>
+        <v>Lo.95.CF6.Y.Pln.1</v>
       </c>
       <c r="C19">
         <f t="shared" si="3"/>
@@ -6749,7 +6863,7 @@
         <v>Y</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I19" s="22">
         <v>1</v>
@@ -6794,27 +6908,27 @@
       </c>
       <c r="Y19" s="6">
         <f t="shared" si="15"/>
-        <v>84.8262</v>
+        <v>96.28919999999998</v>
       </c>
       <c r="Z19" s="6">
         <f t="shared" si="15"/>
-        <v>81.384024857142876</v>
+        <v>95.704587000000018</v>
       </c>
       <c r="AA19" s="6">
         <f t="shared" si="15"/>
-        <v>80.280301714285713</v>
+        <v>97.573055999999994</v>
       </c>
       <c r="AB19" s="6">
         <f t="shared" si="15"/>
-        <v>83.863307999999989</v>
+        <v>115.84507799999999</v>
       </c>
       <c r="AC19" s="6">
         <f t="shared" si="15"/>
-        <v>91.376485714285707</v>
+        <v>142.1412</v>
       </c>
       <c r="AD19" s="6">
         <f t="shared" si="15"/>
-        <v>97.914980914285707</v>
+        <v>165.0259332</v>
       </c>
       <c r="AE19" t="s">
         <v>17</v>
@@ -6830,7 +6944,7 @@
       </c>
       <c r="B20" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF6.Y.Y.1</v>
+        <v>Hi.95.CF6.Y.Pln.1</v>
       </c>
       <c r="C20">
         <f t="shared" si="3"/>
@@ -6841,7 +6955,7 @@
         <v>Hi</v>
       </c>
       <c r="E20">
-        <f t="shared" ref="E20:E72" si="17">E16</f>
+        <f t="shared" ref="E20:E83" si="17">E16</f>
         <v>95</v>
       </c>
       <c r="F20" t="s">
@@ -6852,7 +6966,7 @@
         <v>Y</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I20" s="22">
         <v>1</v>
@@ -6897,27 +7011,27 @@
       </c>
       <c r="Y20" s="6">
         <f t="shared" si="15"/>
-        <v>126.02749714285714</v>
+        <v>143.05823999999998</v>
       </c>
       <c r="Z20" s="6">
         <f t="shared" si="15"/>
-        <v>133.17385885714287</v>
+        <v>156.60750600000003</v>
       </c>
       <c r="AA20" s="6">
         <f t="shared" si="15"/>
-        <v>132.96424971428573</v>
+        <v>161.60537400000001</v>
       </c>
       <c r="AB20" s="6">
         <f t="shared" si="15"/>
-        <v>140.673936</v>
+        <v>194.320776</v>
       </c>
       <c r="AC20" s="6">
         <f t="shared" si="15"/>
-        <v>147.38142857142856</v>
+        <v>229.26</v>
       </c>
       <c r="AD20" s="6">
         <f t="shared" si="15"/>
-        <v>151.61029302857142</v>
+        <v>255.52402559999999</v>
       </c>
       <c r="AE20" t="s">
         <v>17</v>
@@ -6933,7 +7047,7 @@
       </c>
       <c r="B21" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF6.N.Y.1</v>
+        <v>Lo.0.CF6.N.Pln.1</v>
       </c>
       <c r="C21">
         <f t="shared" si="3"/>
@@ -6955,7 +7069,7 @@
         <v>N</v>
       </c>
       <c r="H21" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I21" s="22">
         <v>1</v>
@@ -7039,7 +7153,7 @@
       </c>
       <c r="B22" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF6.N.Y.1</v>
+        <v>Hi.0.CF6.N.Pln.1</v>
       </c>
       <c r="C22">
         <f t="shared" si="3"/>
@@ -7061,7 +7175,7 @@
         <v>N</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I22" s="22">
         <v>1</v>
@@ -7075,27 +7189,27 @@
       </c>
       <c r="Y22" s="6">
         <f t="shared" si="19"/>
-        <v>29.214274285714311</v>
+        <v>33.471960000000024</v>
       </c>
       <c r="Z22" s="6">
         <f t="shared" si="19"/>
-        <v>29.767773428571417</v>
+        <v>35.409206999999981</v>
       </c>
       <c r="AA22" s="6">
         <f t="shared" si="19"/>
-        <v>35.338791428571426</v>
+        <v>43.444770000000005</v>
       </c>
       <c r="AB22" s="6">
         <f t="shared" si="19"/>
-        <v>43.696956</v>
+        <v>61.235345999999993</v>
       </c>
       <c r="AC22" s="6">
         <f t="shared" si="19"/>
-        <v>53.712342857142858</v>
+        <v>84.826199999999972</v>
       </c>
       <c r="AD22" s="6">
         <f t="shared" si="19"/>
-        <v>64.036903200000012</v>
+        <v>109.4991612</v>
       </c>
       <c r="AE22" t="s">
         <v>17</v>
@@ -7111,7 +7225,7 @@
       </c>
       <c r="B23" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF6.N.Y.1</v>
+        <v>Lo.95.CF6.N.Pln.1</v>
       </c>
       <c r="C23">
         <f t="shared" si="3"/>
@@ -7133,7 +7247,7 @@
         <v>N</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I23" s="22">
         <v>1</v>
@@ -7152,7 +7266,7 @@
       </c>
       <c r="B24" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF6.N.Y.1</v>
+        <v>Hi.95.CF6.N.Pln.1</v>
       </c>
       <c r="C24">
         <f t="shared" si="3"/>
@@ -7174,7 +7288,7 @@
         <v>N</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I24" s="22">
         <v>1</v>
@@ -7192,23 +7306,23 @@
       </c>
       <c r="O24" s="11">
         <f t="shared" si="20"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P24" s="11">
         <f t="shared" si="20"/>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="Q24" s="11">
         <f t="shared" si="20"/>
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="R24" s="11">
         <f t="shared" si="20"/>
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="S24" s="11">
         <f t="shared" si="20"/>
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="W24" t="s">
         <v>28</v>
@@ -7218,23 +7332,23 @@
       </c>
       <c r="Z24" s="11">
         <f>O24/1000</f>
-        <v>3.0000000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="AA24" s="11">
         <f>P24/1000</f>
-        <v>3.5000000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="AB24" s="11">
         <f>Q24/1000</f>
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="AC24" s="11">
         <f>R24/1000</f>
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="AD24" s="11">
         <f>S24/1000</f>
-        <v>9.5000000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="AE24" t="s">
         <v>29</v>
@@ -7250,7 +7364,7 @@
       </c>
       <c r="B25" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF1.Y.Y.0.25</v>
+        <v>Lo.0.CF1.Y.Pln.0.25</v>
       </c>
       <c r="C25">
         <f t="shared" si="3"/>
@@ -7273,7 +7387,7 @@
         <v>Y</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I25" s="23">
         <v>0.25</v>
@@ -7289,7 +7403,7 @@
       </c>
       <c r="B26" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF1.Y.Y.0.25</v>
+        <v>Hi.0.CF1.Y.Pln.0.25</v>
       </c>
       <c r="C26">
         <f t="shared" si="3"/>
@@ -7304,7 +7418,7 @@
         <v>0</v>
       </c>
       <c r="F26" t="str">
-        <f t="shared" ref="F26:F72" si="21">F10</f>
+        <f t="shared" ref="F26:F89" si="21">F10</f>
         <v>CF1</v>
       </c>
       <c r="G26" t="str">
@@ -7312,7 +7426,7 @@
         <v>Y</v>
       </c>
       <c r="H26" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I26" s="23">
         <v>0.25</v>
@@ -7331,7 +7445,7 @@
       </c>
       <c r="B27" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF1.Y.Y.0.25</v>
+        <v>Lo.95.CF1.Y.Pln.0.25</v>
       </c>
       <c r="C27">
         <f t="shared" si="3"/>
@@ -7354,7 +7468,7 @@
         <v>Y</v>
       </c>
       <c r="H27" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I27" s="23">
         <v>0.25</v>
@@ -7407,7 +7521,7 @@
       </c>
       <c r="B28" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF1.Y.Y.0.25</v>
+        <v>Hi.95.CF1.Y.Pln.0.25</v>
       </c>
       <c r="C28">
         <f t="shared" si="3"/>
@@ -7430,7 +7544,7 @@
         <v>Y</v>
       </c>
       <c r="H28" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I28" s="23">
         <v>0.25</v>
@@ -7468,7 +7582,7 @@
       </c>
       <c r="B29" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF1.N.Y.0.25</v>
+        <v>Lo.0.CF1.N.Pln.0.25</v>
       </c>
       <c r="C29">
         <f t="shared" si="3"/>
@@ -7491,7 +7605,7 @@
         <v>N</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I29" s="23">
         <v>0.25</v>
@@ -7529,7 +7643,7 @@
       </c>
       <c r="B30" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF1.N.Y.0.25</v>
+        <v>Hi.0.CF1.N.Pln.0.25</v>
       </c>
       <c r="C30">
         <f t="shared" si="3"/>
@@ -7552,7 +7666,7 @@
         <v>N</v>
       </c>
       <c r="H30" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I30" s="23">
         <v>0.25</v>
@@ -7568,7 +7682,7 @@
       </c>
       <c r="B31" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF1.N.Y.0.25</v>
+        <v>Lo.95.CF1.N.Pln.0.25</v>
       </c>
       <c r="C31">
         <f t="shared" si="3"/>
@@ -7591,7 +7705,7 @@
         <v>N</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I31" s="23">
         <v>0.25</v>
@@ -7607,7 +7721,7 @@
       </c>
       <c r="B32" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF1.N.Y.0.25</v>
+        <v>Hi.95.CF1.N.Pln.0.25</v>
       </c>
       <c r="C32">
         <f t="shared" si="3"/>
@@ -7630,14 +7744,14 @@
         <v>N</v>
       </c>
       <c r="H32" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I32" s="23">
         <v>0.25</v>
       </c>
       <c r="W32" s="5" t="str">
         <f>IF($G$5="N","~TFM_UPD","DEF correction active")</f>
-        <v>~TFM_UPD</v>
+        <v>DEF correction active</v>
       </c>
       <c r="AN32" s="10">
         <f t="shared" si="9"/>
@@ -7650,7 +7764,7 @@
       </c>
       <c r="B33" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF6.Y.Y.0.25</v>
+        <v>Lo.0.CF6.Y.Pln.0.25</v>
       </c>
       <c r="C33">
         <f t="shared" si="3"/>
@@ -7673,7 +7787,7 @@
         <v>Y</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I33" s="23">
         <v>0.25</v>
@@ -7701,7 +7815,7 @@
       </c>
       <c r="B34" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF6.Y.Y.0.25</v>
+        <v>Hi.0.CF6.Y.Pln.0.25</v>
       </c>
       <c r="C34">
         <f t="shared" si="3"/>
@@ -7724,7 +7838,7 @@
         <v>Y</v>
       </c>
       <c r="H34" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I34" s="23">
         <v>0.25</v>
@@ -7752,7 +7866,7 @@
       </c>
       <c r="B35" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF6.Y.Y.0.25</v>
+        <v>Lo.95.CF6.Y.Pln.0.25</v>
       </c>
       <c r="C35">
         <f t="shared" si="3"/>
@@ -7775,7 +7889,7 @@
         <v>Y</v>
       </c>
       <c r="H35" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I35" s="23">
         <v>0.25</v>
@@ -7791,7 +7905,7 @@
       </c>
       <c r="B36" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF6.Y.Y.0.25</v>
+        <v>Hi.95.CF6.Y.Pln.0.25</v>
       </c>
       <c r="C36">
         <f t="shared" si="3"/>
@@ -7814,7 +7928,7 @@
         <v>Y</v>
       </c>
       <c r="H36" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I36" s="23">
         <v>0.25</v>
@@ -7833,7 +7947,7 @@
       </c>
       <c r="B37" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF6.N.Y.0.25</v>
+        <v>Lo.0.CF6.N.Pln.0.25</v>
       </c>
       <c r="C37">
         <f t="shared" si="3"/>
@@ -7856,7 +7970,7 @@
         <v>N</v>
       </c>
       <c r="H37" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I37" s="23">
         <v>0.25</v>
@@ -7897,7 +8011,7 @@
       </c>
       <c r="W37" s="5" t="str">
         <f>IF($G$5="N","~TFM_INS: limtype=LO","DEF correction active")</f>
-        <v>~TFM_INS: limtype=LO</v>
+        <v>DEF correction active</v>
       </c>
       <c r="AN37" s="10">
         <f t="shared" si="9"/>
@@ -7910,7 +8024,7 @@
       </c>
       <c r="B38" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF6.N.Y.0.25</v>
+        <v>Hi.0.CF6.N.Pln.0.25</v>
       </c>
       <c r="C38">
         <f t="shared" si="3"/>
@@ -7933,7 +8047,7 @@
         <v>N</v>
       </c>
       <c r="H38" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I38" s="23">
         <v>0.25</v>
@@ -7995,7 +8109,7 @@
       </c>
       <c r="B39" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF6.N.Y.0.25</v>
+        <v>Lo.95.CF6.N.Pln.0.25</v>
       </c>
       <c r="C39">
         <f t="shared" si="3"/>
@@ -8018,7 +8132,7 @@
         <v>N</v>
       </c>
       <c r="H39" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I39" s="23">
         <v>0.25</v>
@@ -8080,7 +8194,7 @@
       </c>
       <c r="B40" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF6.N.Y.0.25</v>
+        <v>Hi.95.CF6.N.Pln.0.25</v>
       </c>
       <c r="C40">
         <f t="shared" si="3"/>
@@ -8103,7 +8217,7 @@
         <v>N</v>
       </c>
       <c r="H40" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I40" s="23">
         <v>0.25</v>
@@ -8162,7 +8276,7 @@
       </c>
       <c r="B41" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF1.Y.Y.2</v>
+        <v>Lo.0.CF1.Y.Pln.2</v>
       </c>
       <c r="C41">
         <f t="shared" si="3"/>
@@ -8185,7 +8299,7 @@
         <v>Y</v>
       </c>
       <c r="H41" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I41" s="23">
         <v>2</v>
@@ -8201,7 +8315,7 @@
       </c>
       <c r="B42" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF1.Y.Y.2</v>
+        <v>Hi.0.CF1.Y.Pln.2</v>
       </c>
       <c r="C42">
         <f t="shared" si="3"/>
@@ -8224,7 +8338,7 @@
         <v>Y</v>
       </c>
       <c r="H42" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I42" s="23">
         <v>2</v>
@@ -8240,7 +8354,7 @@
       </c>
       <c r="B43" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF1.Y.Y.2</v>
+        <v>Lo.95.CF1.Y.Pln.2</v>
       </c>
       <c r="C43">
         <f t="shared" si="3"/>
@@ -8263,7 +8377,7 @@
         <v>Y</v>
       </c>
       <c r="H43" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I43" s="23">
         <v>2</v>
@@ -8282,7 +8396,7 @@
       </c>
       <c r="B44" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF1.Y.Y.2</v>
+        <v>Hi.95.CF1.Y.Pln.2</v>
       </c>
       <c r="C44">
         <f t="shared" si="3"/>
@@ -8305,7 +8419,7 @@
         <v>Y</v>
       </c>
       <c r="H44" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I44" s="23">
         <v>2</v>
@@ -8360,7 +8474,7 @@
       </c>
       <c r="B45" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF1.N.Y.2</v>
+        <v>Lo.0.CF1.N.Pln.2</v>
       </c>
       <c r="C45">
         <f t="shared" si="3"/>
@@ -8383,7 +8497,7 @@
         <v>N</v>
       </c>
       <c r="H45" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I45" s="23">
         <v>2</v>
@@ -8442,7 +8556,7 @@
       </c>
       <c r="B46" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF1.N.Y.2</v>
+        <v>Hi.0.CF1.N.Pln.2</v>
       </c>
       <c r="C46">
         <f t="shared" si="3"/>
@@ -8465,7 +8579,7 @@
         <v>N</v>
       </c>
       <c r="H46" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I46" s="23">
         <v>2</v>
@@ -8524,7 +8638,7 @@
       </c>
       <c r="B47" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF1.N.Y.2</v>
+        <v>Lo.95.CF1.N.Pln.2</v>
       </c>
       <c r="C47">
         <f t="shared" si="3"/>
@@ -8547,7 +8661,7 @@
         <v>N</v>
       </c>
       <c r="H47" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I47" s="23">
         <v>2</v>
@@ -8606,7 +8720,7 @@
       </c>
       <c r="B48" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF1.N.Y.2</v>
+        <v>Hi.95.CF1.N.Pln.2</v>
       </c>
       <c r="C48">
         <f t="shared" si="3"/>
@@ -8629,7 +8743,7 @@
         <v>N</v>
       </c>
       <c r="H48" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I48" s="23">
         <v>2</v>
@@ -8668,7 +8782,7 @@
       </c>
       <c r="B49" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF6.Y.Y.2</v>
+        <v>Lo.0.CF6.Y.Pln.2</v>
       </c>
       <c r="C49">
         <f t="shared" si="3"/>
@@ -8691,7 +8805,7 @@
         <v>Y</v>
       </c>
       <c r="H49" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I49" s="23">
         <v>2</v>
@@ -8707,7 +8821,7 @@
       </c>
       <c r="B50" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF6.Y.Y.2</v>
+        <v>Hi.0.CF6.Y.Pln.2</v>
       </c>
       <c r="C50">
         <f t="shared" si="3"/>
@@ -8730,7 +8844,7 @@
         <v>Y</v>
       </c>
       <c r="H50" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I50" s="23">
         <v>2</v>
@@ -8746,7 +8860,7 @@
       </c>
       <c r="B51" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF6.Y.Y.2</v>
+        <v>Lo.95.CF6.Y.Pln.2</v>
       </c>
       <c r="C51">
         <f t="shared" si="3"/>
@@ -8769,13 +8883,16 @@
         <v>Y</v>
       </c>
       <c r="H51" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I51" s="23">
         <v>2</v>
       </c>
+      <c r="U51" t="s">
+        <v>135</v>
+      </c>
       <c r="W51" s="5" t="str">
-        <f>IF($H$5="N","~TFM_INS: limtype=LO","GAS available")</f>
+        <f>IF($U$51="N","~TFM_INS: limtype=LO","GAS available")</f>
         <v>GAS available</v>
       </c>
       <c r="AN51" s="10">
@@ -8789,7 +8906,7 @@
       </c>
       <c r="B52" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF6.Y.Y.2</v>
+        <v>Hi.95.CF6.Y.Pln.2</v>
       </c>
       <c r="C52">
         <f t="shared" si="3"/>
@@ -8812,7 +8929,7 @@
         <v>Y</v>
       </c>
       <c r="H52" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I52" s="23">
         <v>2</v>
@@ -8843,7 +8960,7 @@
       </c>
       <c r="B53" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.0.CF6.N.Y.2</v>
+        <v>Lo.0.CF6.N.Pln.2</v>
       </c>
       <c r="C53">
         <f t="shared" si="3"/>
@@ -8866,7 +8983,7 @@
         <v>N</v>
       </c>
       <c r="H53" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I53" s="23">
         <v>2</v>
@@ -8894,7 +9011,7 @@
       </c>
       <c r="B54" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.0.CF6.N.Y.2</v>
+        <v>Hi.0.CF6.N.Pln.2</v>
       </c>
       <c r="C54">
         <f t="shared" si="3"/>
@@ -8917,7 +9034,7 @@
         <v>N</v>
       </c>
       <c r="H54" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I54" s="23">
         <v>2</v>
@@ -8933,7 +9050,7 @@
       </c>
       <c r="B55" t="str">
         <f t="shared" si="2"/>
-        <v>Lo.95.CF6.N.Y.2</v>
+        <v>Lo.95.CF6.N.Pln.2</v>
       </c>
       <c r="C55">
         <f t="shared" si="3"/>
@@ -8956,7 +9073,7 @@
         <v>N</v>
       </c>
       <c r="H55" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I55" s="23">
         <v>2</v>
@@ -8972,7 +9089,7 @@
       </c>
       <c r="B56" t="str">
         <f t="shared" si="2"/>
-        <v>Hi.95.CF6.N.Y.2</v>
+        <v>Hi.95.CF6.N.Pln.2</v>
       </c>
       <c r="C56">
         <f t="shared" si="3"/>
@@ -8995,7 +9112,7 @@
         <v>N</v>
       </c>
       <c r="H56" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I56" s="23">
         <v>2</v>
@@ -9011,7 +9128,7 @@
       </c>
       <c r="B57" t="str">
         <f t="shared" ref="B57:B72" si="30">_xlfn.TEXTJOIN(".",TRUE,D57:I57)</f>
-        <v>Lo.0.CF1.Y.Y.0.1</v>
+        <v>Lo.0.CF1.Y.Pln.0.1</v>
       </c>
       <c r="C57">
         <f t="shared" si="3"/>
@@ -9034,7 +9151,7 @@
         <v>Y</v>
       </c>
       <c r="H57" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I57" s="23">
         <v>0.1</v>
@@ -9062,7 +9179,7 @@
       </c>
       <c r="B58" t="str">
         <f t="shared" si="30"/>
-        <v>Hi.0.CF1.Y.Y.0.1</v>
+        <v>Hi.0.CF1.Y.Pln.0.1</v>
       </c>
       <c r="C58">
         <f t="shared" si="3"/>
@@ -9085,7 +9202,7 @@
         <v>Y</v>
       </c>
       <c r="H58" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I58" s="23">
         <v>0.1</v>
@@ -9131,7 +9248,7 @@
       </c>
       <c r="B59" t="str">
         <f t="shared" si="30"/>
-        <v>Lo.95.CF1.Y.Y.0.1</v>
+        <v>Lo.95.CF1.Y.Pln.0.1</v>
       </c>
       <c r="C59">
         <f t="shared" si="3"/>
@@ -9154,7 +9271,7 @@
         <v>Y</v>
       </c>
       <c r="H59" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I59" s="23">
         <v>0.1</v>
@@ -9199,7 +9316,7 @@
       </c>
       <c r="B60" t="str">
         <f t="shared" si="30"/>
-        <v>Hi.95.CF1.Y.Y.0.1</v>
+        <v>Hi.95.CF1.Y.Pln.0.1</v>
       </c>
       <c r="C60">
         <f t="shared" si="3"/>
@@ -9222,7 +9339,7 @@
         <v>Y</v>
       </c>
       <c r="H60" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I60" s="23">
         <v>0.1</v>
@@ -9238,7 +9355,7 @@
       </c>
       <c r="B61" t="str">
         <f t="shared" si="30"/>
-        <v>Lo.0.CF1.N.Y.0.1</v>
+        <v>Lo.0.CF1.N.Pln.0.1</v>
       </c>
       <c r="C61">
         <f t="shared" si="3"/>
@@ -9261,7 +9378,7 @@
         <v>N</v>
       </c>
       <c r="H61" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I61" s="23">
         <v>0.1</v>
@@ -9271,13 +9388,13 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" spans="1:40" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:40" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A62">
         <v>5</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="30"/>
-        <v>Hi.0.CF1.N.Y.0.1</v>
+        <v>Hi.0.CF1.N.Pln.0.1</v>
       </c>
       <c r="C62">
         <f t="shared" si="3"/>
@@ -9300,23 +9417,27 @@
         <v>N</v>
       </c>
       <c r="H62" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I62" s="23">
         <v>0.1</v>
+      </c>
+      <c r="W62" s="5" t="str">
+        <f>IF($H$5&lt;&gt;"Pln","~TFM_UPD","Coal plants retire as per plan")</f>
+        <v>~TFM_UPD</v>
       </c>
       <c r="AN62" s="10">
         <f t="shared" si="9"/>
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:40" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:40" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A63">
         <v>5</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="30"/>
-        <v>Lo.95.CF1.N.Y.0.1</v>
+        <v>Lo.95.CF1.N.Pln.0.1</v>
       </c>
       <c r="C63">
         <f t="shared" si="3"/>
@@ -9339,10 +9460,22 @@
         <v>N</v>
       </c>
       <c r="H63" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I63" s="23">
         <v>0.1</v>
+      </c>
+      <c r="W63" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="X63" s="24" t="s">
+        <v>150</v>
+      </c>
+      <c r="Y63" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="Z63" s="24" t="s">
+        <v>163</v>
       </c>
       <c r="AN63" s="10">
         <f t="shared" si="9"/>
@@ -9355,7 +9488,7 @@
       </c>
       <c r="B64" t="str">
         <f t="shared" si="30"/>
-        <v>Hi.95.CF1.N.Y.0.1</v>
+        <v>Hi.95.CF1.N.Pln.0.1</v>
       </c>
       <c r="C64">
         <f t="shared" si="3"/>
@@ -9378,10 +9511,20 @@
         <v>N</v>
       </c>
       <c r="H64" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I64" s="23">
         <v>0.1</v>
+      </c>
+      <c r="W64" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="X64" s="26"/>
+      <c r="Y64" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="Z64" s="25" t="s">
+        <v>164</v>
       </c>
       <c r="AN64" s="10">
         <f t="shared" si="9"/>
@@ -9394,7 +9537,7 @@
       </c>
       <c r="B65" t="str">
         <f t="shared" si="30"/>
-        <v>Lo.0.CF6.Y.Y.0.1</v>
+        <v>Lo.0.CF6.Y.Pln.0.1</v>
       </c>
       <c r="C65">
         <f t="shared" si="3"/>
@@ -9417,7 +9560,7 @@
         <v>Y</v>
       </c>
       <c r="H65" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I65" s="23">
         <v>0.1</v>
@@ -9433,7 +9576,7 @@
       </c>
       <c r="B66" t="str">
         <f t="shared" si="30"/>
-        <v>Hi.0.CF6.Y.Y.0.1</v>
+        <v>Hi.0.CF6.Y.Pln.0.1</v>
       </c>
       <c r="C66">
         <f t="shared" si="3"/>
@@ -9456,7 +9599,7 @@
         <v>Y</v>
       </c>
       <c r="H66" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I66" s="23">
         <v>0.1</v>
@@ -9472,7 +9615,7 @@
       </c>
       <c r="B67" t="str">
         <f t="shared" si="30"/>
-        <v>Lo.95.CF6.Y.Y.0.1</v>
+        <v>Lo.95.CF6.Y.Pln.0.1</v>
       </c>
       <c r="C67">
         <f t="shared" si="3"/>
@@ -9495,7 +9638,7 @@
         <v>Y</v>
       </c>
       <c r="H67" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I67" s="23">
         <v>0.1</v>
@@ -9511,7 +9654,7 @@
       </c>
       <c r="B68" t="str">
         <f t="shared" si="30"/>
-        <v>Hi.95.CF6.Y.Y.0.1</v>
+        <v>Hi.95.CF6.Y.Pln.0.1</v>
       </c>
       <c r="C68">
         <f t="shared" si="3"/>
@@ -9534,7 +9677,7 @@
         <v>Y</v>
       </c>
       <c r="H68" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I68" s="23">
         <v>0.1</v>
@@ -9550,7 +9693,7 @@
       </c>
       <c r="B69" t="str">
         <f t="shared" si="30"/>
-        <v>Lo.0.CF6.N.Y.0.1</v>
+        <v>Lo.0.CF6.N.Pln.0.1</v>
       </c>
       <c r="C69">
         <f t="shared" si="3"/>
@@ -9573,7 +9716,7 @@
         <v>N</v>
       </c>
       <c r="H69" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I69" s="23">
         <v>0.1</v>
@@ -9589,7 +9732,7 @@
       </c>
       <c r="B70" t="str">
         <f t="shared" si="30"/>
-        <v>Hi.0.CF6.N.Y.0.1</v>
+        <v>Hi.0.CF6.N.Pln.0.1</v>
       </c>
       <c r="C70">
         <f t="shared" si="3"/>
@@ -9612,7 +9755,7 @@
         <v>N</v>
       </c>
       <c r="H70" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I70" s="23">
         <v>0.1</v>
@@ -9628,7 +9771,7 @@
       </c>
       <c r="B71" t="str">
         <f t="shared" si="30"/>
-        <v>Lo.95.CF6.N.Y.0.1</v>
+        <v>Lo.95.CF6.N.Pln.0.1</v>
       </c>
       <c r="C71">
         <f t="shared" si="3"/>
@@ -9651,7 +9794,7 @@
         <v>N</v>
       </c>
       <c r="H71" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I71" s="23">
         <v>0.1</v>
@@ -9667,7 +9810,7 @@
       </c>
       <c r="B72" t="str">
         <f t="shared" si="30"/>
-        <v>Hi.95.CF6.N.Y.0.1</v>
+        <v>Hi.95.CF6.N.Pln.0.1</v>
       </c>
       <c r="C72">
         <f t="shared" si="3"/>
@@ -9690,7 +9833,7 @@
         <v>N</v>
       </c>
       <c r="H72" s="15" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="I72" s="23">
         <v>0.1</v>
@@ -9701,39 +9844,2267 @@
       </c>
     </row>
     <row r="73" spans="1:40" x14ac:dyDescent="0.45">
+      <c r="A73">
+        <v>5</v>
+      </c>
+      <c r="B73" t="str">
+        <f t="shared" ref="B73:B136" si="31">_xlfn.TEXTJOIN(".",TRUE,D73:I73)</f>
+        <v>Lo.0.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C73">
+        <f t="shared" si="3"/>
+        <v>65</v>
+      </c>
+      <c r="D73" t="str">
+        <f t="shared" si="4"/>
+        <v>Lo</v>
+      </c>
+      <c r="E73">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F73" t="str">
+        <f t="shared" si="21"/>
+        <v>CF1</v>
+      </c>
+      <c r="G73" t="str">
+        <f t="shared" si="14"/>
+        <v>Y</v>
+      </c>
+      <c r="H73" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I73" s="23">
+        <v>0.1</v>
+      </c>
       <c r="AN73" s="10">
         <f t="shared" si="9"/>
         <v>13</v>
       </c>
     </row>
     <row r="74" spans="1:40" x14ac:dyDescent="0.45">
+      <c r="A74">
+        <v>5</v>
+      </c>
+      <c r="B74" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C74">
+        <f t="shared" si="3"/>
+        <v>66</v>
+      </c>
+      <c r="D74" t="str">
+        <f t="shared" si="4"/>
+        <v>Hi</v>
+      </c>
+      <c r="E74">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F74" t="str">
+        <f t="shared" si="21"/>
+        <v>CF1</v>
+      </c>
+      <c r="G74" t="str">
+        <f t="shared" si="14"/>
+        <v>Y</v>
+      </c>
+      <c r="H74" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I74" s="23">
+        <v>0.1</v>
+      </c>
       <c r="AN74" s="10">
         <f t="shared" si="9"/>
         <v>14</v>
       </c>
     </row>
     <row r="75" spans="1:40" x14ac:dyDescent="0.45">
+      <c r="A75">
+        <v>5</v>
+      </c>
+      <c r="B75" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C75">
+        <f t="shared" ref="C75:C138" si="32">C74+1</f>
+        <v>67</v>
+      </c>
+      <c r="D75" t="str">
+        <f t="shared" si="4"/>
+        <v>Lo</v>
+      </c>
+      <c r="E75">
+        <f t="shared" si="17"/>
+        <v>95</v>
+      </c>
+      <c r="F75" t="str">
+        <f t="shared" si="21"/>
+        <v>CF1</v>
+      </c>
+      <c r="G75" t="str">
+        <f t="shared" si="14"/>
+        <v>Y</v>
+      </c>
+      <c r="H75" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I75" s="23">
+        <v>0.1</v>
+      </c>
       <c r="AN75" s="10">
         <f t="shared" si="9"/>
         <v>14</v>
       </c>
     </row>
     <row r="76" spans="1:40" x14ac:dyDescent="0.45">
+      <c r="A76">
+        <v>5</v>
+      </c>
+      <c r="B76" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C76">
+        <f t="shared" si="32"/>
+        <v>68</v>
+      </c>
+      <c r="D76" t="str">
+        <f t="shared" ref="D76:D139" si="33">D74</f>
+        <v>Hi</v>
+      </c>
+      <c r="E76">
+        <f t="shared" si="17"/>
+        <v>95</v>
+      </c>
+      <c r="F76" t="str">
+        <f t="shared" si="21"/>
+        <v>CF1</v>
+      </c>
+      <c r="G76" t="str">
+        <f t="shared" si="14"/>
+        <v>Y</v>
+      </c>
+      <c r="H76" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I76" s="23">
+        <v>0.1</v>
+      </c>
       <c r="AN76" s="10">
         <f t="shared" si="9"/>
         <v>14</v>
       </c>
     </row>
     <row r="77" spans="1:40" x14ac:dyDescent="0.45">
+      <c r="A77">
+        <v>5</v>
+      </c>
+      <c r="B77" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C77">
+        <f t="shared" si="32"/>
+        <v>69</v>
+      </c>
+      <c r="D77" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E77">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F77" t="str">
+        <f t="shared" si="21"/>
+        <v>CF1</v>
+      </c>
+      <c r="G77" t="str">
+        <f t="shared" si="14"/>
+        <v>N</v>
+      </c>
+      <c r="H77" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I77" s="23">
+        <v>0.1</v>
+      </c>
       <c r="AN77" s="10">
         <f t="shared" si="9"/>
         <v>14</v>
       </c>
     </row>
     <row r="78" spans="1:40" x14ac:dyDescent="0.45">
+      <c r="A78">
+        <v>5</v>
+      </c>
+      <c r="B78" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C78">
+        <f t="shared" si="32"/>
+        <v>70</v>
+      </c>
+      <c r="D78" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E78">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F78" t="str">
+        <f t="shared" si="21"/>
+        <v>CF1</v>
+      </c>
+      <c r="G78" t="str">
+        <f t="shared" si="14"/>
+        <v>N</v>
+      </c>
+      <c r="H78" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I78" s="23">
+        <v>0.1</v>
+      </c>
       <c r="AN78" s="10">
         <f t="shared" si="9"/>
         <v>14</v>
+      </c>
+    </row>
+    <row r="79" spans="1:40" x14ac:dyDescent="0.45">
+      <c r="A79">
+        <v>5</v>
+      </c>
+      <c r="B79" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C79">
+        <f t="shared" si="32"/>
+        <v>71</v>
+      </c>
+      <c r="D79" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E79">
+        <f t="shared" si="17"/>
+        <v>95</v>
+      </c>
+      <c r="F79" t="str">
+        <f t="shared" si="21"/>
+        <v>CF1</v>
+      </c>
+      <c r="G79" t="str">
+        <f t="shared" si="14"/>
+        <v>N</v>
+      </c>
+      <c r="H79" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I79" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:40" x14ac:dyDescent="0.45">
+      <c r="A80">
+        <v>5</v>
+      </c>
+      <c r="B80" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C80">
+        <f t="shared" si="32"/>
+        <v>72</v>
+      </c>
+      <c r="D80" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E80">
+        <f t="shared" si="17"/>
+        <v>95</v>
+      </c>
+      <c r="F80" t="str">
+        <f t="shared" si="21"/>
+        <v>CF1</v>
+      </c>
+      <c r="G80" t="str">
+        <f t="shared" si="14"/>
+        <v>N</v>
+      </c>
+      <c r="H80" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I80" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A81">
+        <v>5</v>
+      </c>
+      <c r="B81" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C81">
+        <f t="shared" si="32"/>
+        <v>73</v>
+      </c>
+      <c r="D81" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E81">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F81" t="str">
+        <f t="shared" si="21"/>
+        <v>CF6</v>
+      </c>
+      <c r="G81" t="str">
+        <f t="shared" si="14"/>
+        <v>Y</v>
+      </c>
+      <c r="H81" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I81" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A82">
+        <v>5</v>
+      </c>
+      <c r="B82" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C82">
+        <f t="shared" si="32"/>
+        <v>74</v>
+      </c>
+      <c r="D82" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E82">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F82" t="str">
+        <f t="shared" si="21"/>
+        <v>CF6</v>
+      </c>
+      <c r="G82" t="str">
+        <f t="shared" ref="G82:G145" si="34">G74</f>
+        <v>Y</v>
+      </c>
+      <c r="H82" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I82" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A83">
+        <v>5</v>
+      </c>
+      <c r="B83" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C83">
+        <f t="shared" si="32"/>
+        <v>75</v>
+      </c>
+      <c r="D83" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E83">
+        <f t="shared" si="17"/>
+        <v>95</v>
+      </c>
+      <c r="F83" t="str">
+        <f t="shared" si="21"/>
+        <v>CF6</v>
+      </c>
+      <c r="G83" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H83" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I83" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A84">
+        <v>5</v>
+      </c>
+      <c r="B84" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C84">
+        <f t="shared" si="32"/>
+        <v>76</v>
+      </c>
+      <c r="D84" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E84">
+        <f t="shared" ref="E84:E147" si="35">E80</f>
+        <v>95</v>
+      </c>
+      <c r="F84" t="str">
+        <f t="shared" si="21"/>
+        <v>CF6</v>
+      </c>
+      <c r="G84" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H84" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I84" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A85">
+        <v>5</v>
+      </c>
+      <c r="B85" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C85">
+        <f t="shared" si="32"/>
+        <v>77</v>
+      </c>
+      <c r="D85" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E85">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F85" t="str">
+        <f t="shared" si="21"/>
+        <v>CF6</v>
+      </c>
+      <c r="G85" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H85" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I85" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A86">
+        <v>5</v>
+      </c>
+      <c r="B86" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C86">
+        <f t="shared" si="32"/>
+        <v>78</v>
+      </c>
+      <c r="D86" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E86">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F86" t="str">
+        <f t="shared" si="21"/>
+        <v>CF6</v>
+      </c>
+      <c r="G86" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H86" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I86" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A87">
+        <v>5</v>
+      </c>
+      <c r="B87" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C87">
+        <f t="shared" si="32"/>
+        <v>79</v>
+      </c>
+      <c r="D87" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E87">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F87" t="str">
+        <f t="shared" si="21"/>
+        <v>CF6</v>
+      </c>
+      <c r="G87" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H87" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I87" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A88">
+        <v>5</v>
+      </c>
+      <c r="B88" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C88">
+        <f t="shared" si="32"/>
+        <v>80</v>
+      </c>
+      <c r="D88" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E88">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F88" t="str">
+        <f t="shared" si="21"/>
+        <v>CF6</v>
+      </c>
+      <c r="G88" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H88" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I88" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A89">
+        <v>5</v>
+      </c>
+      <c r="B89" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C89">
+        <f t="shared" si="32"/>
+        <v>81</v>
+      </c>
+      <c r="D89" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E89">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F89" t="str">
+        <f t="shared" si="21"/>
+        <v>CF1</v>
+      </c>
+      <c r="G89" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H89" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I89" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A90">
+        <v>5</v>
+      </c>
+      <c r="B90" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C90">
+        <f t="shared" si="32"/>
+        <v>82</v>
+      </c>
+      <c r="D90" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E90">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F90" t="str">
+        <f t="shared" ref="F90:F153" si="36">F74</f>
+        <v>CF1</v>
+      </c>
+      <c r="G90" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H90" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I90" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A91">
+        <v>5</v>
+      </c>
+      <c r="B91" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C91">
+        <f t="shared" si="32"/>
+        <v>83</v>
+      </c>
+      <c r="D91" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E91">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F91" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G91" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H91" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I91" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A92">
+        <v>5</v>
+      </c>
+      <c r="B92" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C92">
+        <f t="shared" si="32"/>
+        <v>84</v>
+      </c>
+      <c r="D92" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E92">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F92" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G92" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H92" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I92" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A93">
+        <v>5</v>
+      </c>
+      <c r="B93" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C93">
+        <f t="shared" si="32"/>
+        <v>85</v>
+      </c>
+      <c r="D93" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E93">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F93" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G93" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H93" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I93" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A94">
+        <v>5</v>
+      </c>
+      <c r="B94" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C94">
+        <f t="shared" si="32"/>
+        <v>86</v>
+      </c>
+      <c r="D94" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E94">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F94" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G94" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H94" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I94" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A95">
+        <v>5</v>
+      </c>
+      <c r="B95" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C95">
+        <f t="shared" si="32"/>
+        <v>87</v>
+      </c>
+      <c r="D95" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E95">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F95" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G95" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H95" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I95" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A96">
+        <v>5</v>
+      </c>
+      <c r="B96" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C96">
+        <f t="shared" si="32"/>
+        <v>88</v>
+      </c>
+      <c r="D96" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E96">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F96" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G96" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H96" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I96" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A97">
+        <v>5</v>
+      </c>
+      <c r="B97" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C97">
+        <f t="shared" si="32"/>
+        <v>89</v>
+      </c>
+      <c r="D97" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E97">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F97" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G97" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H97" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I97" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A98">
+        <v>5</v>
+      </c>
+      <c r="B98" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C98">
+        <f t="shared" si="32"/>
+        <v>90</v>
+      </c>
+      <c r="D98" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E98">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F98" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G98" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H98" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I98" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A99">
+        <v>5</v>
+      </c>
+      <c r="B99" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C99">
+        <f t="shared" si="32"/>
+        <v>91</v>
+      </c>
+      <c r="D99" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E99">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F99" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G99" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H99" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I99" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A100">
+        <v>5</v>
+      </c>
+      <c r="B100" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C100">
+        <f t="shared" si="32"/>
+        <v>92</v>
+      </c>
+      <c r="D100" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E100">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F100" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G100" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H100" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I100" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A101">
+        <v>5</v>
+      </c>
+      <c r="B101" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C101">
+        <f t="shared" si="32"/>
+        <v>93</v>
+      </c>
+      <c r="D101" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E101">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F101" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G101" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H101" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I101" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A102">
+        <v>5</v>
+      </c>
+      <c r="B102" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C102">
+        <f t="shared" si="32"/>
+        <v>94</v>
+      </c>
+      <c r="D102" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E102">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F102" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G102" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H102" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I102" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A103">
+        <v>5</v>
+      </c>
+      <c r="B103" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C103">
+        <f t="shared" si="32"/>
+        <v>95</v>
+      </c>
+      <c r="D103" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E103">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F103" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G103" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H103" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I103" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A104">
+        <v>5</v>
+      </c>
+      <c r="B104" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C104">
+        <f t="shared" si="32"/>
+        <v>96</v>
+      </c>
+      <c r="D104" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E104">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F104" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G104" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H104" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I104" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A105">
+        <v>5</v>
+      </c>
+      <c r="B105" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C105">
+        <f t="shared" si="32"/>
+        <v>97</v>
+      </c>
+      <c r="D105" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E105">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F105" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G105" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H105" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I105" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A106">
+        <v>5</v>
+      </c>
+      <c r="B106" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C106">
+        <f t="shared" si="32"/>
+        <v>98</v>
+      </c>
+      <c r="D106" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E106">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F106" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G106" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H106" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I106" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A107">
+        <v>5</v>
+      </c>
+      <c r="B107" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C107">
+        <f t="shared" si="32"/>
+        <v>99</v>
+      </c>
+      <c r="D107" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E107">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F107" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G107" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H107" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I107" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A108">
+        <v>5</v>
+      </c>
+      <c r="B108" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C108">
+        <f t="shared" si="32"/>
+        <v>100</v>
+      </c>
+      <c r="D108" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E108">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F108" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G108" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H108" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I108" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A109">
+        <v>5</v>
+      </c>
+      <c r="B109" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C109">
+        <f t="shared" si="32"/>
+        <v>101</v>
+      </c>
+      <c r="D109" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E109">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F109" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G109" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H109" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I109" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A110">
+        <v>5</v>
+      </c>
+      <c r="B110" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C110">
+        <f t="shared" si="32"/>
+        <v>102</v>
+      </c>
+      <c r="D110" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E110">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F110" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G110" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H110" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I110" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A111">
+        <v>5</v>
+      </c>
+      <c r="B111" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C111">
+        <f t="shared" si="32"/>
+        <v>103</v>
+      </c>
+      <c r="D111" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E111">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F111" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G111" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H111" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I111" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A112">
+        <v>5</v>
+      </c>
+      <c r="B112" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C112">
+        <f t="shared" si="32"/>
+        <v>104</v>
+      </c>
+      <c r="D112" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E112">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F112" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G112" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H112" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I112" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A113">
+        <v>5</v>
+      </c>
+      <c r="B113" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C113">
+        <f t="shared" si="32"/>
+        <v>105</v>
+      </c>
+      <c r="D113" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E113">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F113" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G113" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H113" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I113" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A114">
+        <v>5</v>
+      </c>
+      <c r="B114" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C114">
+        <f t="shared" si="32"/>
+        <v>106</v>
+      </c>
+      <c r="D114" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E114">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F114" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G114" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H114" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I114" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A115">
+        <v>5</v>
+      </c>
+      <c r="B115" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C115">
+        <f t="shared" si="32"/>
+        <v>107</v>
+      </c>
+      <c r="D115" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E115">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F115" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G115" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H115" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I115" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A116">
+        <v>5</v>
+      </c>
+      <c r="B116" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C116">
+        <f t="shared" si="32"/>
+        <v>108</v>
+      </c>
+      <c r="D116" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E116">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F116" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G116" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H116" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I116" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A117">
+        <v>5</v>
+      </c>
+      <c r="B117" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C117">
+        <f t="shared" si="32"/>
+        <v>109</v>
+      </c>
+      <c r="D117" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E117">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F117" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G117" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H117" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I117" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A118">
+        <v>5</v>
+      </c>
+      <c r="B118" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C118">
+        <f t="shared" si="32"/>
+        <v>110</v>
+      </c>
+      <c r="D118" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E118">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F118" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G118" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H118" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I118" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A119">
+        <v>5</v>
+      </c>
+      <c r="B119" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C119">
+        <f t="shared" si="32"/>
+        <v>111</v>
+      </c>
+      <c r="D119" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E119">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F119" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G119" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H119" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I119" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A120">
+        <v>5</v>
+      </c>
+      <c r="B120" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C120">
+        <f t="shared" si="32"/>
+        <v>112</v>
+      </c>
+      <c r="D120" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E120">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F120" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G120" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H120" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I120" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A121">
+        <v>5</v>
+      </c>
+      <c r="B121" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C121">
+        <f t="shared" si="32"/>
+        <v>113</v>
+      </c>
+      <c r="D121" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E121">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F121" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G121" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H121" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I121" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A122">
+        <v>5</v>
+      </c>
+      <c r="B122" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C122">
+        <f t="shared" si="32"/>
+        <v>114</v>
+      </c>
+      <c r="D122" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E122">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F122" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G122" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H122" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I122" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A123">
+        <v>5</v>
+      </c>
+      <c r="B123" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C123">
+        <f t="shared" si="32"/>
+        <v>115</v>
+      </c>
+      <c r="D123" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E123">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F123" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G123" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H123" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I123" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A124">
+        <v>5</v>
+      </c>
+      <c r="B124" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF1.Y.Eco.0.1</v>
+      </c>
+      <c r="C124">
+        <f t="shared" si="32"/>
+        <v>116</v>
+      </c>
+      <c r="D124" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E124">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F124" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G124" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H124" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I124" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A125">
+        <v>5</v>
+      </c>
+      <c r="B125" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C125">
+        <f t="shared" si="32"/>
+        <v>117</v>
+      </c>
+      <c r="D125" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E125">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F125" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G125" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H125" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I125" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A126">
+        <v>5</v>
+      </c>
+      <c r="B126" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C126">
+        <f t="shared" si="32"/>
+        <v>118</v>
+      </c>
+      <c r="D126" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E126">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F126" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G126" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H126" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I126" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A127">
+        <v>5</v>
+      </c>
+      <c r="B127" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C127">
+        <f t="shared" si="32"/>
+        <v>119</v>
+      </c>
+      <c r="D127" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E127">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F127" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G127" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H127" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I127" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A128">
+        <v>5</v>
+      </c>
+      <c r="B128" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF1.N.Eco.0.1</v>
+      </c>
+      <c r="C128">
+        <f t="shared" si="32"/>
+        <v>120</v>
+      </c>
+      <c r="D128" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E128">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F128" t="str">
+        <f t="shared" si="36"/>
+        <v>CF1</v>
+      </c>
+      <c r="G128" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H128" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I128" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A129">
+        <v>5</v>
+      </c>
+      <c r="B129" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C129">
+        <f t="shared" si="32"/>
+        <v>121</v>
+      </c>
+      <c r="D129" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E129">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F129" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G129" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H129" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I129" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A130">
+        <v>5</v>
+      </c>
+      <c r="B130" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C130">
+        <f t="shared" si="32"/>
+        <v>122</v>
+      </c>
+      <c r="D130" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E130">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F130" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G130" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H130" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I130" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A131">
+        <v>5</v>
+      </c>
+      <c r="B131" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C131">
+        <f t="shared" si="32"/>
+        <v>123</v>
+      </c>
+      <c r="D131" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E131">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F131" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G131" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H131" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I131" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A132">
+        <v>5</v>
+      </c>
+      <c r="B132" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF6.Y.Eco.0.1</v>
+      </c>
+      <c r="C132">
+        <f t="shared" si="32"/>
+        <v>124</v>
+      </c>
+      <c r="D132" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E132">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F132" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G132" t="str">
+        <f t="shared" si="34"/>
+        <v>Y</v>
+      </c>
+      <c r="H132" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I132" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A133">
+        <v>5</v>
+      </c>
+      <c r="B133" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.0.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C133">
+        <f t="shared" si="32"/>
+        <v>125</v>
+      </c>
+      <c r="D133" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E133">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F133" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G133" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H133" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I133" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A134">
+        <v>5</v>
+      </c>
+      <c r="B134" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.0.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C134">
+        <f t="shared" si="32"/>
+        <v>126</v>
+      </c>
+      <c r="D134" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E134">
+        <f t="shared" si="35"/>
+        <v>0</v>
+      </c>
+      <c r="F134" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G134" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H134" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I134" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A135">
+        <v>5</v>
+      </c>
+      <c r="B135" t="str">
+        <f t="shared" si="31"/>
+        <v>Lo.95.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C135">
+        <f t="shared" si="32"/>
+        <v>127</v>
+      </c>
+      <c r="D135" t="str">
+        <f t="shared" si="33"/>
+        <v>Lo</v>
+      </c>
+      <c r="E135">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F135" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G135" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H135" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I135" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A136">
+        <v>5</v>
+      </c>
+      <c r="B136" t="str">
+        <f t="shared" si="31"/>
+        <v>Hi.95.CF6.N.Eco.0.1</v>
+      </c>
+      <c r="C136">
+        <f t="shared" si="32"/>
+        <v>128</v>
+      </c>
+      <c r="D136" t="str">
+        <f t="shared" si="33"/>
+        <v>Hi</v>
+      </c>
+      <c r="E136">
+        <f t="shared" si="35"/>
+        <v>95</v>
+      </c>
+      <c r="F136" t="str">
+        <f t="shared" si="36"/>
+        <v>CF6</v>
+      </c>
+      <c r="G136" t="str">
+        <f t="shared" si="34"/>
+        <v>N</v>
+      </c>
+      <c r="H136" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="I136" s="23">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>